<commit_message>
feat: add format-aware barcode workflows across SKU create/import/print
</commit_message>
<xml_diff>
--- a/public/sku-import-template.xlsx
+++ b/public/sku-import-template.xlsx
@@ -397,52 +397,59 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F2"/>
   <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="36.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="36.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" customWidth="1"/>
+    <col min="6" max="6" width="36.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>barcode_format</v>
+      </c>
+      <c r="B1" t="str">
         <v>gtin</v>
       </c>
-      <c r="B1" t="str">
+      <c r="C1" t="str">
         <v>name</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>lot</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>price</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>logo_url</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>ean13</v>
+      </c>
+      <c r="B2" t="str">
         <v>5901234123457</v>
       </c>
-      <c r="B2" t="str">
+      <c r="C2" t="str">
         <v>Example Organic Oat Milk 1L</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>LOT-2024-A</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>4.99</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>